<commit_message>
Rebuild Sun Life social sheet from verified sunlife.com.vn data with sources
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR1qVnPwb7hxUbF4akMpvt
</commit_message>
<xml_diff>
--- a/SunLife_Kich_ban_Social.xlsx
+++ b/SunLife_Kich_ban_Social.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,10 +30,13 @@
       <sz val="14"/>
     </font>
     <font>
+      <i val="1"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -43,6 +46,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFC20E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE9E7"/>
       </patternFill>
     </fill>
   </fills>
@@ -72,17 +80,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -450,17 +462,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="3" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="85" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="3" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -469,14 +482,19 @@
           <t>THÔNG TIN TẠO SOCIAL - SUN LIFE VIỆT NAM</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>DOANH NGHIỆP CUNG CẤP THÔNG TIN SAU:</t>
         </is>
       </c>
     </row>
     <row r="2" ht="75" customHeight="1">
-      <c r="F2" s="3" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Dữ liệu lấy từ sunlife.com.vn (xem cột Nguồn). Ô tô đỏ = cần KH cung cấp.</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>1. Hệ thống social là list các tài khoản social như: tumblr, pinterest... Cần thông tin input như bảng mẫu để tạo tài khoản.
 2. Định hướng: Tạo dưới tên thương hiệu để tăng tín hiệu social, liên kết các tài khoản và share bài để hỗ trợ SEO.</t>
@@ -484,669 +502,765 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Thông tin public trên social</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Nội dung chi tiết</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Nguồn</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Thông tin tài khoản</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Nội dung</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="5" t="n">
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Tên doanh nghiệp - Đầy đủ</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Công ty TNHH Bảo hiểm Nhân thọ Sun Life Việt Nam</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Username</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>sunlifevietnam</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="5" t="n">
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Đề xuất (trùng tên Facebook/Youtube chính thức)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Tên doanh nghiệp - Thương hiệu</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Sun Life Việt Nam</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Tên hiển thị</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Sun Life Việt Nam</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="5" t="n">
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Lĩnh vực kinh doanh</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Bảo hiểm nhân thọ (bảo vệ, sức khỏe, tiết kiệm, đầu tư, hưu trí)</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Bảo hiểm nhân thọ (khách hàng cá nhân và doanh nghiệp; tiên phong lĩnh vực bảo hiểm hưu trí)</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>KH/team SEO cấp email riêng</t>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>Team SEO cấp email riêng</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Địa chỉ</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Tầng 29, Tòa nhà Vietcombank, 5 Công Trường Mê Linh, Phường Bến Nghé, Quận 1, TP. Hồ Chí Minh</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>ok – Sau sáp nhập hành chính 7/2025: Phường Sài Gòn, TP.HCM. Cần thống nhất 1 dạng địa chỉ trên mọi social</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Tầng 29, Tòa nhà Vietcombank Tower, số 05 Công trường Mê Linh, phường Sài Gòn, Thành phố Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>ok – Địa chỉ trụ sở theo trang Liên hệ. Chi nhánh: Hà Nội – Tầng 22 Tòa nhà Capital Place, 29 Liễu Giai, Phường Ngọc Hà, Hà Nội; Đà Nẵng – Tòa nhà Nexus, Số 75-77-79 Xô Viết Nghệ Tĩnh, Phường Cẩm Lệ, TP. Đà Nẵng</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Password</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>KH/team SEO đặt</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>Team SEO đặt</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="6" t="inlineStr"/>
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Zipcode</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>700000</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Mã bưu chính chung TP.HCM (không lấy từ website)</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Zip code</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>700000</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="5" t="n">
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Số điện thoại</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Hotline: 1800 1786
-Tổng đài: (028) 6298 5888
-Fax: (028) 6298 5999</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Tổng đài CSKH: 1800 1786 (miễn cước)
+Điện thoại: (028) 6298 5888</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>Độ tuổi</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr"/>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="5" t="n">
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>dichvu.khachhang@sunlife.com</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Dichvu.Khachhang@sunlife.com</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Giới tính</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Khác</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="150" customHeight="1">
-      <c r="A11" s="5" t="n">
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Lịch sử hoạt động</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>- 01/2013: Thành lập liên doanh PVI Sun Life giữa Tổng CTCP Bảo hiểm PVI (51%) và Sun Life Assurance Company of Canada (49%) – Giấy phép số 68 GP/KDBH do Bộ Tài chính cấp ngày 24/01/2013
-- 01/2016: Tập đoàn Sun Life nâng tỷ lệ sở hữu lên 75%
-- 11/2016: Sun Life mua lại toàn bộ 25% vốn còn lại, đổi tên thành Công ty TNHH Bảo hiểm Nhân thọ Sun Life Việt Nam (100% vốn Canada)
-- 2025: Tăng vốn điều lệ lên 18.434 tỷ đồng; ra mắt 7 sản phẩm mới; chi trả 608 tỷ đồng quyền lợi bảo hiểm (tăng 26%)
-- 03/2026: Tăng vốn điều lệ lên 18.909 tỷ đồng, vào top 3 thị trường về quy mô vốn</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>- 2013: Sun Life đặt chân đến thị trường Việt Nam thông qua liên doanh Bảo hiểm Nhân thọ PVI Sun Life
+- 11/2016: Tập đoàn Sun Life hoàn tất nhận chuyển nhượng 25% cổ phần còn lại; công ty trở thành 100% vốn Sun Life với thương hiệu Sun Life Việt Nam
+- 2026: Được Bộ Tài chính chấp thuận tăng vốn điều lệ lên 18.909 tỷ đồng</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/
+https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2016/tap-doan-tai-chinh-sun-life-hoan-tat-thuong-vu-chuyen-nhuong-25-co-phan-con-lai-tu-cong-ty-pvi-sun-life
+https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2026/sun-life-viet-nam-tang-von-dieu-le-len-18909-ty-dong/</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Ngày sinh/Ngày thành lập</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>24/01/2013</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Ngày cấp giấy phép PVI Sun Life</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="5" t="n">
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>Website chỉ ghi năm 2013 – ngày cụ thể cần KH cung cấp</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Thời gian hoạt động</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>8:30 - 17:30, Thứ 2 - Thứ 6</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Cần KH xác nhận ngày làm việc</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Tổng đài 1800 1786 – chuyên viên hỗ trợ: 8:00 - 18:00, Thứ 2 - Thứ 6 (tổng đài tự động 24/7)
+Trung tâm Dịch vụ Khách hàng: Thứ 2 - Thứ 6: 8:30 - 12:00 và 13:00 - 17:30; Thứ 7: 8:30 - 12:00</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/tong-dai-cham-soc-khach-hang/
+https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/mang-luoi-trung-tam-dich-vu-khach-hang/</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="5" t="n">
+      <c r="A13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Bằng cấp, giải thưởng, chứng nhận...</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>- Giấy phép thành lập và hoạt động số 68 GP/KDBH (Bộ Tài chính, 24/01/2013)
-- Công ty Bảo hiểm Nhân thọ có Dịch vụ Khách hàng tốt nhất Việt Nam 2024 (Tạp chí International Finance)
-- Chứng nhận Great Place To Work® 4 năm liên tiếp (2022–2025)</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>- Công ty Bảo hiểm Nhân thọ có Dịch vụ Khách hàng tốt nhất Việt Nam 2024
+- Great Place To Work® 2022–2025</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>ok – Danh sách đầy đủ xem trang Các giải thưởng</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/cac-giai-thuong/
+https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2023/noi-lam-viec-tot-2023/</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Logo - Avatar</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Lấy từ Facebook: https://www.facebook.com/SunLifeVietnam/photos</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="5" t="n">
+      <c r="H13" s="6" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>Lấy logo chính thức từ website/Facebook https://www.facebook.com/SunLifeVietnam</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Khách hàng nổi bật (nếu có)</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr"/>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Chưa có dữ liệu công khai</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr"/>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Cần KH cung cấp</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>Banner</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr"/>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>Lấy ảnh bìa Facebook https://www.facebook.com/SunLifeVietnam/</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="5" t="n">
+      <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>Lấy ảnh bìa Facebook https://www.facebook.com/SunLifeVietnam</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Đối tác tiêu biểu (nếu có)</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Đối tác ngân hàng phân phối bảo hiểm (bancassurance), VD: ACB</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Cần KH xác nhận</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Ngân hàng TMCP Á Châu (ACB) – thỏa thuận hợp tác độc quyền phân phối sản phẩm bảo hiểm nhân thọ kéo dài 15 năm (công bố năm 2020)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2020/sun-life-viet-nam-va-acb-thoa-thuan-doc-quyen-phan-phoi-bao-hiem-nhan-tho/</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>Kết nối với chúng tôi qua:</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Website: https://www.sunlife.com.vn/vn/
-Facebook: https://www.facebook.com/SunLifeVietnam/
-Youtube: https://www.youtube.com/sunlifevietnam</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="5" t="n">
+Facebook: https://www.facebook.com/SunLifeVietnam
+Youtube: https://www.youtube.com/c/SunLifeVietnam
+Instagram: https://www.instagram.com/sunlifevn/</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="5" t="n">
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Social chính</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Facebook: https://www.facebook.com/SunLifeVietnam/
-Youtube: https://www.youtube.com/sunlifevietnam</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>ok – Chưa tìm thấy LinkedIn/TikTok/Zalo chính thức, cần KH bổ sung</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="5" t="n">
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Facebook: https://www.facebook.com/SunLifeVietnam
+Youtube: https://www.youtube.com/c/SunLifeVietnam
+Instagram: https://www.instagram.com/sunlifevn/
+Zalo Official Account: Sun Life Việt Nam</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>ok – Chưa có link Zalo OA/LinkedIn/TikTok, cần KH cung cấp</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/dich-vu-khach-hang/chuong-trinh-khuyen-mai/2025/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Slogan</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Life's brighter under the sun (Cuộc sống tươi sáng hơn dưới ánh mặt trời)</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Slogan Tập đoàn – cần KH xác nhận slogan tiếng Việt</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="165" customHeight="1">
-      <c r="A19" s="5" t="n">
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Tài chính cho mình. Lạc quan do mình</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Thông điệp chiến dịch thương hiệu trên website – cần KH xác nhận slogan chính thức</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2024/lac-quan-tai-chinh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="180" customHeight="1">
+      <c r="A19" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Bio ngắn</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Sun Life Việt Nam là công ty bảo hiểm nhân thọ 100% vốn Tập đoàn Sun Life (Canada), tiên phong và dẫn đầu thị trường bảo hiểm hưu trí tự nguyện tại Việt Nam.
-Địa chỉ: Tầng 29, Tòa nhà Vietcombank, 5 Công Trường Mê Linh, Phường Bến Nghé, Quận 1, TP. Hồ Chí Minh
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Sun Life Việt Nam là công ty bảo hiểm nhân thọ 100% vốn từ Tập đoàn Sun Life (Canada), tiên phong và dẫn đầu thị trường trong lĩnh vực bảo hiểm hưu trí tại Việt Nam.
+Địa chỉ: Tầng 29, Tòa nhà Vietcombank Tower, số 05 Công trường Mê Linh, phường Sài Gòn, Thành phố Hồ Chí Minh
 Hotline: 1800 1786
 Website: https://www.sunlife.com.vn/vn/
-Email: dichvu.khachhang@sunlife.com
-Facebook: https://www.facebook.com/SunLifeVietnam/
-Youtube: https://www.youtube.com/sunlifevietnam
-#SunLifeVietnam #BaohiemnhanthoSunLife #BaohiemhuutriSunLife #SunLife</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
+Email: Dichvu.Khachhang@sunlife.com
+Facebook: https://www.facebook.com/SunLifeVietnam
+Youtube: https://www.youtube.com/c/SunLifeVietnam
+Instagram: https://www.instagram.com/sunlifevn/
+#SunLifeVietnam #SunLife #BaoHiemNhanTho #BaoHiemHuuTri</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Viết lại từ dữ kiện trên website; hashtag do team SEO đề xuất</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
         </is>
       </c>
     </row>
     <row r="20" ht="240" customHeight="1">
-      <c r="A20" s="5" t="n">
+      <c r="A20" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Bio trung bình</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Sun Life Việt Nam (Công ty TNHH Bảo hiểm Nhân thọ Sun Life Việt Nam) là thành viên của Tập đoàn Sun Life – tổ chức dịch vụ tài chính quốc tế hàng đầu có trụ sở tại Canada với hơn 150 năm kinh nghiệm. Là doanh nghiệp tiên phong và dẫn đầu lĩnh vực bảo hiểm hưu trí tự nguyện, Sun Life Việt Nam cung cấp các giải pháp bảo hiểm bảo vệ, sức khỏe, tiết kiệm, đầu tư và hưu trí cho khách hàng cá nhân và doanh nghiệp. Chúng tôi cam kết giúp khách hàng đạt được sự an toàn tài chính trọn đời và sống khỏe mạnh hơn.
-Địa chỉ: Tầng 29, Tòa nhà Vietcombank, 5 Công Trường Mê Linh, Phường Bến Nghé, Quận 1, TP. Hồ Chí Minh
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Sun Life Việt Nam là công ty bảo hiểm nhân thọ 100% vốn từ Tập đoàn Sun Life (Canada) – tổ chức dịch vụ tài chính quốc tế hàng đầu với kinh nghiệm hoạt động trên 157 năm. Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn, đồng thời là công ty tiên phong và dẫn đầu thị trường trong lĩnh vực bảo hiểm hưu trí, phục vụ cả Khách hàng cá nhân và doanh nghiệp tại Việt Nam.
+Địa chỉ: Tầng 29, Tòa nhà Vietcombank Tower, số 05 Công trường Mê Linh, phường Sài Gòn, Thành phố Hồ Chí Minh
 Hotline: 1800 1786
 Website: https://www.sunlife.com.vn/vn/
-Email: dichvu.khachhang@sunlife.com
-Facebook: https://www.facebook.com/SunLifeVietnam/
-Youtube: https://www.youtube.com/sunlifevietnam
-#SunLifeVietnam #BaohiemnhanthoSunLife #BaohiemhuutriSunLife #SunLife</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="450" customHeight="1">
-      <c r="A21" s="5" t="n">
+Email: Dichvu.Khachhang@sunlife.com
+Facebook: https://www.facebook.com/SunLifeVietnam
+Youtube: https://www.youtube.com/c/SunLifeVietnam
+Instagram: https://www.instagram.com/sunlifevn/
+#SunLifeVietnam #SunLife #BaoHiemNhanTho #BaoHiemHuuTri</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Viết lại từ dữ kiện trên website; hashtag do team SEO đề xuất</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="360" customHeight="1">
+      <c r="A21" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Bio dài + Có link social</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Công ty TNHH Bảo hiểm Nhân thọ Sun Life Việt Nam là công ty bảo hiểm nhân thọ 100% vốn đầu tư từ Tập đoàn Sun Life (Canada) – tổ chức dịch vụ tài chính quốc tế hàng đầu với hơn 150 năm kinh nghiệm, quản lý tổng tài sản 1,6 nghìn tỷ đô la Canada (tính đến 31/12/2025). Tiền thân là liên doanh PVI Sun Life được cấp phép năm 2013, công ty chính thức mang tên Sun Life Việt Nam từ năm 2016 khi Tập đoàn Sun Life sở hữu 100% vốn.
-Sun Life Việt Nam là doanh nghiệp tiên phong và dẫn đầu thị trường bảo hiểm hưu trí tự nguyện với hơn 70% thị phần trong 5 năm liên tiếp; Quỹ Hưu trí tự nguyện đạt gần 4.500 tỷ đồng tài sản năm 2025. Với vốn điều lệ 18.909 tỷ đồng (2026), Sun Life Việt Nam thuộc top 3 doanh nghiệp bảo hiểm nhân thọ có quy mô vốn lớn nhất thị trường. Danh mục sản phẩm đa dạng gồm bảo hiểm liên kết đơn vị (SUN – Vì Nhà Mình, SUN – Khí Chất), bảo hiểm tử kỳ (SUN – Vững Hành Trình), bảo hiểm sức khỏe và bảo vệ thế hệ mới (Sống Chất 2.0, Sống An 2.0, Sống Vững, Sống Chắc) cùng giải pháp hưu trí và phúc lợi cho doanh nghiệp.
-Với mục đích "Giúp khách hàng đạt được sự an toàn tài chính trọn đời và sống khỏe mạnh hơn", Sun Life Việt Nam không ngừng chuyển đổi số, phát triển đa kênh phân phối và nâng cao trải nghiệm khách hàng – được ghi nhận qua giải thưởng "Công ty Bảo hiểm Nhân thọ có Dịch vụ Khách hàng tốt nhất Việt Nam 2024" và chứng nhận Great Place To Work® nhiều năm liền.
-Địa chỉ: Tầng 29, Tòa nhà Vietcombank, 5 Công Trường Mê Linh, Phường Bến Nghé, Quận 1, TP. Hồ Chí Minh
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Sun Life Việt Nam là công ty bảo hiểm nhân thọ 100% vốn từ Tập đoàn Sun Life (Canada). Tập đoàn Sun Life có trụ sở tại Canada, là tổ chức dịch vụ tài chính quốc tế hàng đầu với kinh nghiệm hoạt động trên 157 năm, có mặt ở nhiều quốc gia trên thế giới; tính đến ngày 31/12/2025, Tập đoàn quản lý tổng tài sản 1,6 nghìn tỷ đô la Canada.
+Năm 2013, Sun Life đặt chân đến thị trường Việt Nam thông qua liên doanh Bảo hiểm Nhân thọ PVI Sun Life. Từ tháng 11/2016, công ty trở thành công ty 100% vốn của Sun Life với thương hiệu Sun Life Việt Nam. Năm 2026, Sun Life Việt Nam được Bộ Tài chính chấp thuận tăng vốn điều lệ lên 18.909 tỷ đồng.
+Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn. Là công ty tiên phong và dẫn đầu thị trường trong lĩnh vực bảo hiểm hưu trí, Sun Life Việt Nam phục vụ cả Khách hàng cá nhân và doanh nghiệp, với các giải pháp như Hưu Trí Sun Life và SUN – Trọn Đời Bình An.
+Địa chỉ: Tầng 29, Tòa nhà Vietcombank Tower, số 05 Công trường Mê Linh, phường Sài Gòn, Thành phố Hồ Chí Minh
 Hotline: 1800 1786
 Website: https://www.sunlife.com.vn/vn/
-Email: dichvu.khachhang@sunlife.com
-Facebook: https://www.facebook.com/SunLifeVietnam/
-Youtube: https://www.youtube.com/sunlifevietnam
-#SunLifeVietnam #BaohiemnhanthoSunLife #BaohiemhuutriSunLife #SunLife</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="180" customHeight="1">
-      <c r="A22" s="5" t="n">
+Email: Dichvu.Khachhang@sunlife.com
+Facebook: https://www.facebook.com/SunLifeVietnam
+Youtube: https://www.youtube.com/c/SunLifeVietnam
+Instagram: https://www.instagram.com/sunlifevn/
+#SunLifeVietnam #SunLife #BaoHiemNhanTho #BaoHiemHuuTri</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Viết lại từ dữ kiện trên website; hashtag do team SEO đề xuất</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/
+https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2026/sun-life-viet-nam-tang-von-dieu-le-len-18909-ty-dong/
+https://www.sunlife.com.vn/vn/doanh-nghiep/giai-phap-huu-tri/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Giá trị cốt lõi</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>- Khách hàng là trọng tâm: Mọi giải pháp hướng tới giúp khách hàng an toàn tài chính trọn đời và sống khỏe mạnh hơn; nâng cao trải nghiệm dịch vụ (giải Dịch vụ khách hàng tốt nhất 2024).
-- Tiên phong hưu trí: Dẫn đầu thị trường bảo hiểm hưu trí tự nguyện (&gt;70% thị phần), đồng hành cùng cá nhân và doanh nghiệp xây dựng tương lai vững vàng.
-- Vững mạnh tài chính &amp; đầu tư dài hạn: Vốn điều lệ 18.909 tỷ đồng, chiến lược đầu tư an toàn, minh bạch.
-- Đổi mới &amp; chuyển đổi số: Tăng tốc số hóa, đa dạng kênh phân phối, tối ưu danh mục sản phẩm.
-- Con người &amp; môi trường làm việc: Great Place To Work® 4 năm liên tiếp.
-- Trách nhiệm cộng đồng: Lan tỏa lối sống khỏe mạnh và kiến thức tài chính đến cộng đồng.</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Tổng hợp từ thông tin công khai – nên đối chiếu trang Về chúng tôi</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="150" customHeight="1">
-      <c r="A23" s="5" t="n">
+      <c r="C22" s="6" t="inlineStr"/>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Cần KH cung cấp – không tìm thấy mục Giá trị cốt lõi của công ty trên website</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Tầm nhìn - Sứ mệnh</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>1. Mục đích (Purpose): Giúp khách hàng đạt được sự an toàn tài chính trọn đời và sống khỏe mạnh hơn.
-2. Tầm nhìn: Trở thành công ty bảo hiểm nhân thọ hàng đầu, dẫn đầu lĩnh vực hưu trí tại Việt Nam.
-3. Sứ mệnh:
-- Đối với khách hàng: Mang đến giải pháp bảo vệ, tiết kiệm, đầu tư và hưu trí toàn diện.
-- Đối với nhân viên &amp; tư vấn viên: Xây dựng môi trường làm việc xuất sắc, phát triển sự nghiệp bền vững.
-- Đối với cộng đồng: Lan tỏa lối sống khỏe mạnh và an toàn tài chính.</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Mục đích lấy từ website; tầm nhìn/sứ mệnh chi tiết cần KH xác nhận</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="165" customHeight="1">
-      <c r="A24" s="5" t="n">
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Mục đích: Giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn.</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Website chỉ nêu Mục đích; Tầm nhìn – Sứ mệnh chi tiết cần kh cung cấp</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="225" customHeight="1">
+      <c r="A24" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Đội ngũ nhân sự</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>1. Hội đồng Thành viên
-- Chủ tịch Hội đồng Thành viên: Ông Randy Lianggara
-2. Ban Điều hành (11 thành viên: Tổng Giám đốc và 10 Phó Tổng Giám đốc)
-- Tổng Giám đốc: Bà Lay Hoon Tan (từ 08/2025)
+- Chủ tịch: Ông Randy Lianggara
+- Phó Chủ tịch: Ông David Gerald Broom
+- Thành viên: Ông Tan Haifeng, Bà Lay Hoon Tan
+2. Ban Điều hành
+- Tổng Giám đốc: Bà Lay Hoon Tan
 - Phó TGĐ Tài chính: Ông Patrick Chow
 - Phó TGĐ Nhân sự: Bà Nguyễn Thu Thủy
-- Phó TGĐ Kênh liên kết Ngân hàng: Ông Nguyễn Việt Dũng
-- Phó TGĐ Pháp chế: Bà Vũ Thị Thúy Hằng
-- Phó TGĐ Dịch vụ Khách hàng: Ông Bùi Hoàng Minh
-3. Kênh phân phối: Đại lý, Bancassurance (liên kết ngân hàng), Nous by Sun Life (tư vấn toàn thời gian), kênh Khách hàng doanh nghiệp</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Cần đối chiếu trang Ban Điều hành mới nhất</t>
+- Phó TGĐ Kênh Đại lý: Ông Budi Darmawan
+- Phó TGĐ Kênh Kinh doanh Liên kết với Ngân hàng: Ông Vũ Tuấn Anh
+- Phó TGĐ Khách hàng Doanh nghiệp: Ông Đào Quốc Bảo
+- Phó TGĐ Nghiệp vụ bảo hiểm: Bà Trần Thị Lý
+- Phó TGĐ Công nghệ và Chuyển đổi Số: Ông Chu Lâm Thái
+- Phó TGĐ Tuân thủ: Bà Trần Thuý Hồng Anh
+- Phó TGĐ Sáng kiến Chiến lược: Ông Phạm Công Kháng</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Theo trang Hội đồng Thành viên &amp; Ban Điều hành – có thể chưa đủ toàn bộ thành viên, nên mở link kiểm tra</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/hoi-dong-thanh-vien/
+https://www.sunlife.com.vn/vn/ve-chung-toi/hoi-dong-thanh-vien/ban-dieu-hanh/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="F2:H2"/>
+  <mergeCells count="3">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="G2:I2"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Apply PM feedback: verbatim website intro in bios, highlight items to ask client
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR1qVnPwb7hxUbF4akMpvt
</commit_message>
<xml_diff>
--- a/SunLife_Kich_ban_Social.xlsx
+++ b/SunLife_Kich_ban_Social.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Kịch bản Social" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cần KH bổ sung" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -50,7 +51,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDE9E7"/>
+        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -80,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -95,6 +96,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -491,7 +498,7 @@
     <row r="2" ht="75" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Dữ liệu lấy từ sunlife.com.vn (xem cột Nguồn). Ô tô đỏ = cần KH cung cấp.</t>
+          <t>Dữ liệu lấy từ sunlife.com.vn (xem cột Nguồn). Dòng tô VÀNG = cần hỏi KH (chi tiết ở tab Cần KH bổ sung).</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -634,7 +641,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Bảo hiểm nhân thọ (khách hàng cá nhân và doanh nghiệp; tiên phong lĩnh vực bảo hiểm hưu trí)</t>
+          <t>Bảo hiểm nhân thọ</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -647,13 +654,13 @@
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr"/>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr"/>
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>Team SEO cấp email riêng</t>
         </is>
@@ -683,13 +690,13 @@
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Password</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr"/>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr"/>
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>Team SEO đặt</t>
         </is>
@@ -830,19 +837,19 @@
 https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2026/sun-life-viet-nam-tang-von-dieu-le-len-18909-ty-dong/</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Ngày sinh/Ngày thành lập</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>2013</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>Website chỉ ghi năm 2013 – ngày cụ thể cần KH cung cấp</t>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Website chỉ ghi năm 2013 – cần KH cung cấp ngày cụ thể</t>
         </is>
       </c>
     </row>
@@ -892,20 +899,20 @@
       <c r="A13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Bằng cấp, giải thưởng, chứng nhận...</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>- Công ty Bảo hiểm Nhân thọ có Dịch vụ Khách hàng tốt nhất Việt Nam 2024
 - Great Place To Work® 2022–2025</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>ok – Danh sách đầy đủ xem trang Các giải thưởng</t>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Cần KH xác nhận danh sách giải thưởng/chứng nhận muốn đưa lên social</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -914,15 +921,15 @@
 https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2023/noi-lam-viec-tot-2023/</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>Logo - Avatar</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr"/>
-      <c r="I13" s="6" t="inlineStr">
-        <is>
-          <t>Lấy logo chính thức từ website/Facebook https://www.facebook.com/SunLifeVietnam</t>
+      <c r="H13" s="7" t="inlineStr"/>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>Cần KH cung cấp file logo gốc</t>
         </is>
       </c>
     </row>
@@ -930,27 +937,27 @@
       <c r="A14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Khách hàng nổi bật (nếu có)</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr"/>
+      <c r="C14" s="7" t="inlineStr"/>
       <c r="D14" s="7" t="inlineStr">
         <is>
           <t>Cần KH cung cấp</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr"/>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>Banner</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr"/>
-      <c r="I14" s="6" t="inlineStr">
-        <is>
-          <t>Lấy ảnh bìa Facebook https://www.facebook.com/SunLifeVietnam</t>
+      <c r="H14" s="7" t="inlineStr"/>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>Cần KH cung cấp file banner</t>
         </is>
       </c>
     </row>
@@ -1022,12 +1029,12 @@
       <c r="A17" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Social chính</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Facebook: https://www.facebook.com/SunLifeVietnam
 Youtube: https://www.youtube.com/c/SunLifeVietnam
@@ -1050,17 +1057,17 @@
       <c r="A18" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Slogan</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Tài chính cho mình. Lạc quan do mình</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>Thông điệp chiến dịch thương hiệu trên website – cần KH xác nhận slogan chính thức</t>
         </is>
@@ -1071,7 +1078,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="180" customHeight="1">
+    <row r="19" ht="195" customHeight="1">
       <c r="A19" s="6" t="n">
         <v>15</v>
       </c>
@@ -1082,7 +1089,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Sun Life Việt Nam là công ty bảo hiểm nhân thọ 100% vốn từ Tập đoàn Sun Life (Canada), tiên phong và dẫn đầu thị trường trong lĩnh vực bảo hiểm hưu trí tại Việt Nam.
+          <t>Sun Life Việt Nam là thành viên của tập đoàn Sun Life (trụ sở tại Canada) – Tổ chức dịch vụ tài chính quốc tế hàng đầu với kinh nghiệm hoạt động trên 157 năm có mặt ở nhiều quốc gia trên thế giới.
 Địa chỉ: Tầng 29, Tòa nhà Vietcombank Tower, số 05 Công trường Mê Linh, phường Sài Gòn, Thành phố Hồ Chí Minh
 Hotline: 1800 1786
 Website: https://www.sunlife.com.vn/vn/
@@ -1095,16 +1102,16 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Viết lại từ dữ kiện trên website; hashtag do team SEO đề xuất</t>
+          <t>Ghép nguyên văn các câu giới thiệu trên website; hashtag do team SEO đề xuất</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="240" customHeight="1">
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="210" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>16</v>
       </c>
@@ -1115,7 +1122,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Sun Life Việt Nam là công ty bảo hiểm nhân thọ 100% vốn từ Tập đoàn Sun Life (Canada) – tổ chức dịch vụ tài chính quốc tế hàng đầu với kinh nghiệm hoạt động trên 157 năm. Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn, đồng thời là công ty tiên phong và dẫn đầu thị trường trong lĩnh vực bảo hiểm hưu trí, phục vụ cả Khách hàng cá nhân và doanh nghiệp tại Việt Nam.
+          <t>Sun Life Việt Nam là thành viên của tập đoàn Sun Life (trụ sở tại Canada) – Tổ chức dịch vụ tài chính quốc tế hàng đầu với kinh nghiệm hoạt động trên 157 năm có mặt ở nhiều quốc gia trên thế giới. Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn.
 Địa chỉ: Tầng 29, Tòa nhà Vietcombank Tower, số 05 Công trường Mê Linh, phường Sài Gòn, Thành phố Hồ Chí Minh
 Hotline: 1800 1786
 Website: https://www.sunlife.com.vn/vn/
@@ -1128,16 +1135,16 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Viết lại từ dữ kiện trên website; hashtag do team SEO đề xuất</t>
+          <t>Ghép nguyên văn các câu giới thiệu trên website; hashtag do team SEO đề xuất</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="360" customHeight="1">
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="330" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>17</v>
       </c>
@@ -1148,9 +1155,9 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Sun Life Việt Nam là công ty bảo hiểm nhân thọ 100% vốn từ Tập đoàn Sun Life (Canada). Tập đoàn Sun Life có trụ sở tại Canada, là tổ chức dịch vụ tài chính quốc tế hàng đầu với kinh nghiệm hoạt động trên 157 năm, có mặt ở nhiều quốc gia trên thế giới; tính đến ngày 31/12/2025, Tập đoàn quản lý tổng tài sản 1,6 nghìn tỷ đô la Canada.
-Năm 2013, Sun Life đặt chân đến thị trường Việt Nam thông qua liên doanh Bảo hiểm Nhân thọ PVI Sun Life. Từ tháng 11/2016, công ty trở thành công ty 100% vốn của Sun Life với thương hiệu Sun Life Việt Nam. Năm 2026, Sun Life Việt Nam được Bộ Tài chính chấp thuận tăng vốn điều lệ lên 18.909 tỷ đồng.
-Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn. Là công ty tiên phong và dẫn đầu thị trường trong lĩnh vực bảo hiểm hưu trí, Sun Life Việt Nam phục vụ cả Khách hàng cá nhân và doanh nghiệp, với các giải pháp như Hưu Trí Sun Life và SUN – Trọn Đời Bình An.
+          <t>Sun Life Việt Nam là thành viên của tập đoàn Sun Life (trụ sở tại Canada) – Tổ chức dịch vụ tài chính quốc tế hàng đầu với kinh nghiệm hoạt động trên 157 năm có mặt ở nhiều quốc gia trên thế giới.
+Năm 2013, Sun Life đặt chân đến thị trường Việt Nam thông qua liên doanh Bảo hiểm Nhân thọ PVI Sun Life, từ tháng 11 năm 2016, trở thành công ty 100% vốn của Sun Life với thương hiệu Sun Life Việt Nam.
+Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn. Sun Life Việt Nam là công ty tiên phong và dẫn đầu thị trường trong lĩnh vực bảo hiểm hưu trí, phục vụ cho cả Khách hàng cá nhân và doanh nghiệp tại Việt Nam.
 Địa chỉ: Tầng 29, Tòa nhà Vietcombank Tower, số 05 Công trường Mê Linh, phường Sài Gòn, Thành phố Hồ Chí Minh
 Hotline: 1800 1786
 Website: https://www.sunlife.com.vn/vn/
@@ -1163,14 +1170,13 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Viết lại từ dữ kiện trên website; hashtag do team SEO đề xuất</t>
+          <t>Ghép nguyên văn các câu giới thiệu trên website; hashtag do team SEO đề xuất</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/
-https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2026/sun-life-viet-nam-tang-von-dieu-le-len-18909-ty-dong/
-https://www.sunlife.com.vn/vn/doanh-nghiep/giai-phap-huu-tri/</t>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/
+https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
         </is>
       </c>
     </row>
@@ -1178,12 +1184,12 @@
       <c r="A22" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Giá trị cốt lõi</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr"/>
+      <c r="C22" s="7" t="inlineStr"/>
       <c r="D22" s="7" t="inlineStr">
         <is>
           <t>Cần KH cung cấp – không tìm thấy mục Giá trị cốt lõi của công ty trên website</t>
@@ -1195,14 +1201,14 @@
       <c r="A23" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Tầm nhìn - Sứ mệnh</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>Mục đích: Giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn.</t>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Mục đích: Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn.</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -1220,12 +1226,12 @@
       <c r="A24" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Đội ngũ nhân sự</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>1. Hội đồng Thành viên
 - Chủ tịch: Ông Randy Lianggara
@@ -1244,7 +1250,7 @@
 - Phó TGĐ Sáng kiến Chiến lược: Ông Phạm Công Kháng</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>Theo trang Hội đồng Thành viên &amp; Ban Điều hành – có thể chưa đủ toàn bộ thành viên, nên mở link kiểm tra</t>
         </is>
@@ -1264,4 +1270,254 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Hạng mục</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Hiện trạng</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Cần KH cung cấp / xác nhận</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Khách hàng nổi bật</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Không có trên website</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>Danh sách khách hàng (doanh nghiệp) tiêu biểu được phép public</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Giá trị cốt lõi</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Không có trên website</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Nội dung giá trị cốt lõi chính thức</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Tầm nhìn - Sứ mệnh</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Website chỉ nêu Mục đích</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Nội dung Tầm nhìn và Sứ mệnh chính thức</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Slogan</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Website chỉ có thông điệp chiến dịch 'Tài chính cho mình. Lạc quan do mình'</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Xác nhận slogan chính thức dùng cho social</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Ngày thành lập</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Website chỉ ghi năm 2013</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Ngày/tháng/năm thành lập chính thức</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Social khác</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Website có Facebook, Youtube, Instagram, Zalo OA (không có link Zalo)</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Link Zalo OA, LinkedIn, TikTok (nếu có)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Giải thưởng, chứng nhận</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Đã lấy 2 giải từ website</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Xác nhận danh sách giải thưởng muốn đưa lên social</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Đội ngũ nhân sự</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Lấy từ trang Hội đồng Thành viên &amp; Ban Điều hành</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Xác nhận danh sách đầy đủ, mới nhất</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Logo - Avatar</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr"/>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>File logo gốc (PNG nền trong, kích thước lớn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Banner</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr"/>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>File banner/ảnh bìa</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Email &amp; Password tạo tài khoản</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr"/>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Team SEO cấp (nội bộ, không hỏi KH)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add client question columns and question list tab to Sun Life social sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR1qVnPwb7hxUbF4akMpvt
</commit_message>
<xml_diff>
--- a/SunLife_Kich_ban_Social.xlsx
+++ b/SunLife_Kich_ban_Social.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Kịch bản Social" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Cần KH bổ sung" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Câu hỏi cho KH" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,8 +36,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +51,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFC20E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -81,11 +90,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -98,12 +109,11 @@
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -469,18 +479,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="85" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="3" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="3" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -489,7 +501,7 @@
           <t>THÔNG TIN TẠO SOCIAL - SUN LIFE VIỆT NAM</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>DOANH NGHIỆP CUNG CẤP THÔNG TIN SAU:</t>
         </is>
@@ -498,10 +510,10 @@
     <row r="2" ht="75" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Dữ liệu lấy từ sunlife.com.vn (xem cột Nguồn). Dòng tô VÀNG = cần hỏi KH (chi tiết ở tab Cần KH bổ sung).</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
+          <t>Dữ liệu lấy từ sunlife.com.vn (xem cột Nguồn).  VÀNG = cần KH bổ sung (chưa có dữ liệu)  |  CAM NHẠT = cần KH xác nhận.  Tổng hợp câu hỏi ở tab 'Câu hỏi cho KH'.</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>1. Hệ thống social là list các tài khoản social như: tumblr, pinterest... Cần thông tin input như bảng mẫu để tạo tài khoản.
 2. Định hướng: Tạo dưới tên thương hiệu để tăng tín hiệu social, liên kết các tài khoản và share bài để hỗ trợ SEO.</t>
@@ -531,22 +543,32 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
+          <t>Câu hỏi cho khách hàng</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
           <t>Nguồn</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Thông tin tài khoản</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>Nội dung</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>Ghi chú</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Câu hỏi cho khách hàng</t>
         </is>
       </c>
     </row>
@@ -569,24 +591,30 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>Username</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>sunlifevietnam</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>Đề xuất (trùng tên Facebook/Youtube chính thức)</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Đồng ý dùng 'sunlifevietnam' làm username? Nếu bị trùng, dùng phương án nào (VD: sunlifevn, sunlife.vietnam)?</t>
         </is>
       </c>
     </row>
@@ -609,32 +637,38 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Tên hiển thị</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>Sun Life Việt Nam</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Xác nhận tên hiển thị 'Sun Life Việt Nam'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Lĩnh vực kinh doanh</t>
         </is>
@@ -644,33 +678,39 @@
           <t>Bảo hiểm nhân thọ</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Lĩnh vực public trên social ghi 'Bảo hiểm nhân thọ' là đủ, hay cần ghi chi tiết hơn (VD: Bảo hiểm nhân thọ &amp; Hưu trí)?</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr"/>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>Team SEO cấp email riêng</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
+      <c r="K6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Địa chỉ</t>
         </is>
@@ -680,31 +720,37 @@
           <t>Tầng 29, Tòa nhà Vietcombank Tower, số 05 Công trường Mê Linh, phường Sài Gòn, Thành phố Hồ Chí Minh</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>ok – Địa chỉ trụ sở theo trang Liên hệ. Chi nhánh: Hà Nội – Tầng 22 Tòa nhà Capital Place, 29 Liễu Giai, Phường Ngọc Hà, Hà Nội; Đà Nẵng – Tòa nhà Nexus, Số 75-77-79 Xô Viết Nghệ Tĩnh, Phường Cẩm Lệ, TP. Đà Nẵng</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Xác nhận dùng địa chỉ trụ sở mới (phường Sài Gòn, TP.HCM) cho mọi tài khoản social? Có cần thêm địa chỉ chi nhánh Hà Nội, Đà Nẵng không?</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Password</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr"/>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>Team SEO đặt</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
+      <c r="K7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="45" customHeight="1">
       <c r="A8" s="6" t="inlineStr"/>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Zipcode</t>
         </is>
@@ -714,33 +760,39 @@
           <t>700000</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Mã bưu chính chung TP.HCM (không lấy từ website)</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr"/>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Zipcode dùng 700000 (mã chung TP.HCM) được không, hay doanh nghiệp có mã bưu chính riêng?</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr"/>
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Zip code</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>700000</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
+      <c r="K8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9" ht="45" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Số điện thoại</t>
         </is>
@@ -751,29 +803,35 @@
 Điện thoại: (028) 6298 5888</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Số chính public trên social là hotline 1800 1786? Có được public thêm số (028) 6298 5888 không?</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>Độ tuổi</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="45" customHeight="1">
       <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
@@ -783,37 +841,43 @@
           <t>Dichvu.Khachhang@sunlife.com</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Email Dichvu.Khachhang@sunlife.com có được public trên social không, hay dùng email khác?</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Giới tính</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>Khác</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
+      <c r="K10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Lịch sử hoạt động</t>
         </is>
@@ -825,31 +889,41 @@
 - 2026: Được Bộ Tài chính chấp thuận tăng vốn điều lệ lên 18.909 tỷ đồng</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Có mốc lịch sử nào khác muốn bổ sung? Có được public thông tin vốn điều lệ 18.909 tỷ đồng không?</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/
 https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2016/tap-doan-tai-chinh-sun-life-hoan-tat-thuong-vu-chuyen-nhuong-25-co-phan-con-lai-tu-cong-ty-pvi-sun-life
 https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2026/sun-life-viet-nam-tang-von-dieu-le-len-18909-ty-dong/</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>Ngày sinh/Ngày thành lập</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>2013</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="J11" s="8" t="inlineStr">
         <is>
           <t>Website chỉ ghi năm 2013 – cần KH cung cấp ngày cụ thể</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>Ngày thành lập chính thức (dd/mm/yyyy) là ngày nào?</t>
         </is>
       </c>
     </row>
@@ -857,7 +931,7 @@
       <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Thời gian hoạt động</t>
         </is>
@@ -868,104 +942,130 @@
 Trung tâm Dịch vụ Khách hàng: Thứ 2 - Thứ 6: 8:30 - 12:00 và 13:00 - 17:30; Thứ 7: 8:30 - 12:00</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Giờ hoạt động public trên social dùng giờ tổng đài (8:00–18:00, T2–T6) hay giờ Trung tâm Dịch vụ Khách hàng (có sáng T7)?</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/tong-dai-cham-soc-khach-hang/
 https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/mang-luoi-trung-tam-dich-vu-khach-hang/</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
+      <c r="K12" s="6" t="inlineStr"/>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Bằng cấp, giải thưởng, chứng nhận...</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>- Công ty Bảo hiểm Nhân thọ có Dịch vụ Khách hàng tốt nhất Việt Nam 2024
 - Great Place To Work® 2022–2025</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>Cần KH xác nhận danh sách giải thưởng/chứng nhận muốn đưa lên social</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Gửi danh sách giải thưởng/chứng nhận chính thức muốn public (tên giải, năm, đơn vị trao).</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/cac-giai-thuong/
 https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2023/noi-lam-viec-tot-2023/</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="H13" s="8" t="inlineStr">
         <is>
           <t>Logo - Avatar</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="8" t="inlineStr">
         <is>
           <t>Cần KH cung cấp file logo gốc</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>Gửi file logo gốc (PNG nền trong, ≥1000px, có bản vuông cho avatar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
       <c r="A14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Khách hàng nổi bật (nếu có)</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr"/>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr"/>
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Cần KH cung cấp</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr"/>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Có khách hàng (doanh nghiệp) tiêu biểu nào được phép công bố trên social không? Nếu có, gửi danh sách.</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr"/>
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>Banner</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr"/>
-      <c r="I14" s="7" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="8" t="inlineStr">
         <is>
           <t>Cần KH cung cấp file banner</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>Gửi banner/ảnh bìa (gợi ý 1500x500px) hoặc đồng ý cho dùng ảnh bìa Facebook hiện tại.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Đối tác tiêu biểu (nếu có)</t>
         </is>
@@ -975,22 +1075,27 @@
           <t>Ngân hàng TMCP Á Châu (ACB) – thỏa thuận hợp tác độc quyền phân phối sản phẩm bảo hiểm nhân thọ kéo dài 15 năm (công bố năm 2020)</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Ngoài ACB, còn đối tác nào (ngân hàng, đối tác chiến lược) muốn đưa lên social không?</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2020/sun-life-viet-nam-va-acb-thoa-thuan-doc-quyen-phan-phoi-bao-hiem-nhan-tho/</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Kết nối với chúng tôi qua:</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>Website: https://www.sunlife.com.vn/vn/
 Facebook: https://www.facebook.com/SunLifeVietnam
@@ -998,11 +1103,12 @@
 Instagram: https://www.instagram.com/sunlifevn/</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
+      <c r="K15" s="6" t="inlineStr"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -1024,17 +1130,18 @@
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr"/>
+      <c r="F16" s="6" t="inlineStr"/>
     </row>
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Social chính</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Facebook: https://www.facebook.com/SunLifeVietnam
 Youtube: https://www.youtube.com/c/SunLifeVietnam
@@ -1042,37 +1149,47 @@
 Zalo Official Account: Sun Life Việt Nam</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>ok – Chưa có link Zalo OA/LinkedIn/TikTok, cần KH cung cấp</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Gửi link Zalo OA, LinkedIn, TikTok (nếu có) và xác nhận link Facebook/Youtube/Instagram chính thức.</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/dich-vu-khach-hang/chuong-trinh-khuyen-mai/2025/</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
+    <row r="18" ht="60" customHeight="1">
       <c r="A18" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Slogan</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Tài chính cho mình. Lạc quan do mình</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Thông điệp chiến dịch thương hiệu trên website – cần KH xác nhận slogan chính thức</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Slogan chính thức của Sun Life Việt Nam là gì? Có dùng thông điệp 'Tài chính cho mình. Lạc quan do mình' làm slogan được không?</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2024/lac-quan-tai-chinh/</t>
         </is>
@@ -1082,7 +1199,7 @@
       <c r="A19" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Bio ngắn</t>
         </is>
@@ -1100,12 +1217,17 @@
 #SunLifeVietnam #SunLife #BaoHiemNhanTho #BaoHiemHuuTri</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>Ghép nguyên văn các câu giới thiệu trên website; hashtag do team SEO đề xuất</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Duyệt nội dung Bio ngắn (câu giới thiệu lấy nguyên văn từ website). Thương hiệu có bộ hashtag chính thức không?</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
         </is>
@@ -1115,7 +1237,7 @@
       <c r="A20" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Bio trung bình</t>
         </is>
@@ -1133,12 +1255,17 @@
 #SunLifeVietnam #SunLife #BaoHiemNhanTho #BaoHiemHuuTri</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>Ghép nguyên văn các câu giới thiệu trên website; hashtag do team SEO đề xuất</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Duyệt nội dung Bio trung bình – có câu nào cần sửa/thêm không?</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
         </is>
@@ -1148,7 +1275,7 @@
       <c r="A21" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Bio dài + Có link social</t>
         </is>
@@ -1168,12 +1295,17 @@
 #SunLifeVietnam #SunLife #BaoHiemNhanTho #BaoHiemHuuTri</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>Ghép nguyên văn các câu giới thiệu trên website; hashtag do team SEO đề xuất</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Duyệt nội dung Bio dài – có muốn bổ sung sản phẩm/thông điệp chủ lực nào không?</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/
 https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
@@ -1184,39 +1316,49 @@
       <c r="A22" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Giá trị cốt lõi</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr"/>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr"/>
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>Cần KH cung cấp – không tìm thấy mục Giá trị cốt lõi của công ty trên website</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23" ht="30" customHeight="1">
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Gửi nội dung Giá trị cốt lõi chính thức của Sun Life Việt Nam.</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23" ht="45" customHeight="1">
       <c r="A23" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Tầm nhìn - Sứ mệnh</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Mục đích: Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn.</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>Website chỉ nêu Mục đích; Tầm nhìn – Sứ mệnh chi tiết cần kh cung cấp</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Gửi nội dung Tầm nhìn, Sứ mệnh chính thức (hay chỉ dùng Mục đích của Tập đoàn như trên website)?</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
         </is>
@@ -1231,7 +1373,7 @@
           <t>Đội ngũ nhân sự</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>1. Hội đồng Thành viên
 - Chủ tịch: Ông Randy Lianggara
@@ -1255,7 +1397,12 @@
           <t>Theo trang Hội đồng Thành viên &amp; Ban Điều hành – có thể chưa đủ toàn bộ thành viên, nên mở link kiểm tra</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Xác nhận danh sách Hội đồng Thành viên &amp; Ban Điều hành mới nhất. Có được public tên lãnh đạo trên social không?</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/hoi-dong-thanh-vien/
 https://www.sunlife.com.vn/vn/ve-chung-toi/hoi-dong-thanh-vien/ban-dieu-hanh/</t>
@@ -1264,9 +1411,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="G2:I2"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="H2:K2"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1278,246 +1425,832 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>DANH SÁCH CÂU HỎI GỬI KHÁCH HÀNG – SUN LIFE VIỆT NAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>KH vui lòng điền vào cột 'Câu trả lời của KH'. VÀNG = cần bổ sung, CAM NHẠT = cần xác nhận.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Nhóm</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Hạng mục</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Hiện trạng</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Cần KH cung cấp / xác nhận</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="8" t="n">
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Dữ liệu hiện có (từ website)</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Câu hỏi cho khách hàng</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Mức độ</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Câu trả lời của KH</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="9" t="inlineStr">
-        <is>
-          <t>Khách hàng nổi bật</t>
-        </is>
-      </c>
-      <c r="C2" s="9" t="inlineStr">
-        <is>
-          <t>Không có trên website</t>
-        </is>
-      </c>
-      <c r="D2" s="9" t="inlineStr">
-        <is>
-          <t>Danh sách khách hàng (doanh nghiệp) tiêu biểu được phép public</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="n">
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Bằng cấp, giải thưởng, chứng nhận...</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>- Công ty Bảo hiểm Nhân thọ có Dịch vụ Khách hàng tốt nhất Việt Nam 2024
+- Great Place To Work® 2022–2025</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Gửi danh sách giải thưởng/chứng nhận chính thức muốn public (tên giải, năm, đơn vị trao).</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Cần bổ sung</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Khách hàng nổi bật (nếu có)</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>(trống)</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Có khách hàng (doanh nghiệp) tiêu biểu nào được phép công bố trên social không? Nếu có, gửi danh sách.</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Cần bổ sung</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Social chính</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Facebook: https://www.facebook.com/SunLifeVietnam
+Youtube: https://www.youtube.com/c/SunLifeVietnam
+Instagram: https://www.instagram.com/sunlifevn/
+Zalo Official Account: Sun Life Việt Nam</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Gửi link Zalo OA, LinkedIn, TikTok (nếu có) và xác nhận link Facebook/Youtube/Instagram chính thức.</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Cần bổ sung</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Slogan</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Tài chính cho mình. Lạc quan do mình</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Slogan chính thức của Sun Life Việt Nam là gì? Có dùng thông điệp 'Tài chính cho mình. Lạc quan do mình' làm slogan được không?</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Cần bổ sung</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Giá trị cốt lõi</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>Không có trên website</t>
-        </is>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>Nội dung giá trị cốt lõi chính thức</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>(trống)</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Gửi nội dung Giá trị cốt lõi chính thức của Sun Life Việt Nam.</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Cần bổ sung</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Tầm nhìn - Sứ mệnh</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>Website chỉ nêu Mục đích</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>Nội dung Tầm nhìn và Sứ mệnh chính thức</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Slogan</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>Website chỉ có thông điệp chiến dịch 'Tài chính cho mình. Lạc quan do mình'</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>Xác nhận slogan chính thức dùng cho social</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Ngày thành lập</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>Website chỉ ghi năm 2013</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Ngày/tháng/năm thành lập chính thức</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>Social khác</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>Website có Facebook, Youtube, Instagram, Zalo OA (không có link Zalo)</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>Link Zalo OA, LinkedIn, TikTok (nếu có)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="n">
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Mục đích: Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Gửi nội dung Tầm nhìn, Sứ mệnh chính thức (hay chỉ dùng Mục đích của Tập đoàn như trên website)?</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Cần bổ sung</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>Giải thưởng, chứng nhận</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Đã lấy 2 giải từ website</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>Xác nhận danh sách giải thưởng muốn đưa lên social</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="n">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Tạo tài khoản</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Ngày sinh/Ngày thành lập</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Ngày thành lập chính thức (dd/mm/yyyy) là ngày nào?</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Cần bổ sung</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Tạo tài khoản</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Logo - Avatar</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>(trống)</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Gửi file logo gốc (PNG nền trong, ≥1000px, có bản vuông cho avatar).</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Cần bổ sung</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Tạo tài khoản</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Banner</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>(trống)</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Gửi banner/ảnh bìa (gợi ý 1500x500px) hoặc đồng ý cho dùng ảnh bìa Facebook hiện tại.</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Cần bổ sung</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Lĩnh vực kinh doanh</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Bảo hiểm nhân thọ</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Lĩnh vực public trên social ghi 'Bảo hiểm nhân thọ' là đủ, hay cần ghi chi tiết hơn (VD: Bảo hiểm nhân thọ &amp; Hưu trí)?</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Cần xác nhận</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Địa chỉ</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Tầng 29, Tòa nhà Vietcombank Tower, số 05 Công trường Mê Linh, phường Sài Gòn, Thành phố Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Xác nhận dùng địa chỉ trụ sở mới (phường Sài Gòn, TP.HCM) cho mọi tài khoản social? Có cần thêm địa chỉ chi nhánh Hà Nội, Đà Nẵng không?</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Cần xác nhận</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Zipcode</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>700000</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Zipcode dùng 700000 (mã chung TP.HCM) được không, hay doanh nghiệp có mã bưu chính riêng?</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Cần xác nhận</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Số điện thoại</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Tổng đài CSKH: 1800 1786 (miễn cước)
+Điện thoại: (028) 6298 5888</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Số chính public trên social là hotline 1800 1786? Có được public thêm số (028) 6298 5888 không?</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Cần xác nhận</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Dichvu.Khachhang@sunlife.com</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Email Dichvu.Khachhang@sunlife.com có được public trên social không, hay dùng email khác?</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Cần xác nhận</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Lịch sử hoạt động</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>- 2013: Sun Life đặt chân đến thị trường Việt Nam thông qua liên doanh Bảo hiểm Nhân thọ PVI Sun Life
+- 11/2016: Tập đoàn Sun Life hoàn tất nhận chuyển nhượng 25% cổ phần còn lại; công ty trở thành 100% vốn Sun Life với thương hiệu Sun Life Việt Nam
+- 2026: Được Bộ Tài chính chấp thuận tăng vốn điều…</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Có mốc lịch sử nào khác muốn bổ sung? Có được public thông tin vốn điều lệ 18.909 tỷ đồng không?</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Cần xác nhận</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Thời gian hoạt động</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Tổng đài 1800 1786 – chuyên viên hỗ trợ: 8:00 - 18:00, Thứ 2 - Thứ 6 (tổng đài tự động 24/7)
+Trung tâm Dịch vụ Khách hàng: Thứ 2 - Thứ 6: 8:30 - 12:00 và 13:00 - 17:30; Thứ 7: 8:30 - 12:00</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Giờ hoạt động public trên social dùng giờ tổng đài (8:00–18:00, T2–T6) hay giờ Trung tâm Dịch vụ Khách hàng (có sáng T7)?</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>Cần xác nhận</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Đối tác tiêu biểu (nếu có)</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Ngân hàng TMCP Á Châu (ACB) – thỏa thuận hợp tác độc quyền phân phối sản phẩm bảo hiểm nhân thọ kéo dài 15 năm (công bố năm 2020)</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Ngoài ACB, còn đối tác nào (ngân hàng, đối tác chiến lược) muốn đưa lên social không?</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>Cần xác nhận</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Bio ngắn</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Sun Life Việt Nam là thành viên của tập đoàn Sun Life (trụ sở tại Canada) – Tổ chức dịch vụ tài chính quốc tế hàng đầu với kinh nghiệm hoạt động trên 157 năm có mặt ở nhiều quốc gia trên thế giới.
+Địa chỉ: Tầng 29, Tòa nhà Vietcombank Tower, số 05 Công trường Mê Linh, phường Sài Gòn, Thành phố Hồ C…</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Duyệt nội dung Bio ngắn (câu giới thiệu lấy nguyên văn từ website). Thương hiệu có bộ hashtag chính thức không?</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Cần xác nhận</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Bio trung bình</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Sun Life Việt Nam là thành viên của tập đoàn Sun Life (trụ sở tại Canada) – Tổ chức dịch vụ tài chính quốc tế hàng đầu với kinh nghiệm hoạt động trên 157 năm có mặt ở nhiều quốc gia trên thế giới. Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng c…</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Duyệt nội dung Bio trung bình – có câu nào cần sửa/thêm không?</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Cần xác nhận</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Bio dài + Có link social</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Sun Life Việt Nam là thành viên của tập đoàn Sun Life (trụ sở tại Canada) – Tổ chức dịch vụ tài chính quốc tế hàng đầu với kinh nghiệm hoạt động trên 157 năm có mặt ở nhiều quốc gia trên thế giới.
+Năm 2013, Sun Life đặt chân đến thị trường Việt Nam thông qua liên doanh Bảo hiểm Nhân thọ PVI Sun Lif…</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Duyệt nội dung Bio dài – có muốn bổ sung sản phẩm/thông điệp chủ lực nào không?</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Cần xác nhận</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Thông tin public</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>Đội ngũ nhân sự</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Lấy từ trang Hội đồng Thành viên &amp; Ban Điều hành</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Xác nhận danh sách đầy đủ, mới nhất</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Logo - Avatar</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr"/>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>File logo gốc (PNG nền trong, kích thước lớn)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Banner</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr"/>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>File banner/ảnh bìa</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>1. Hội đồng Thành viên
+- Chủ tịch: Ông Randy Lianggara
+- Phó Chủ tịch: Ông David Gerald Broom
+- Thành viên: Ông Tan Haifeng, Bà Lay Hoon Tan
+2. Ban Điều hành
+- Tổng Giám đốc: Bà Lay Hoon Tan
+- Phó TGĐ Tài chính: Ông Patrick Chow
+- Phó TGĐ Nhân sự: Bà Nguyễn Thu Thủy
+- Phó TGĐ Kênh Đại lý: Ông Budi D…</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Xác nhận danh sách Hội đồng Thành viên &amp; Ban Điều hành mới nhất. Có được public tên lãnh đạo trên social không?</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Cần xác nhận</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Tạo tài khoản</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Username</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>sunlifevietnam</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Đồng ý dùng 'sunlifevietnam' làm username? Nếu bị trùng, dùng phương án nào (VD: sunlifevn, sunlife.vietnam)?</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Cần xác nhận</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Tạo tài khoản</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Tên hiển thị</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Sun Life Việt Nam</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Xác nhận tên hiển thị 'Sun Life Việt Nam'.</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Cần xác nhận</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Nội bộ SEO</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>Email &amp; Password tạo tài khoản</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr"/>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Team SEO cấp (nội bộ, không hỏi KH)</t>
-        </is>
-      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>(trống)</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Team SEO tự cấp – không gửi KH</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr"/>
+      <c r="G27" s="6" t="inlineStr"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Place source link column next to notes; add sources for account table
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR1qVnPwb7hxUbF4akMpvt
</commit_message>
<xml_diff>
--- a/SunLife_Kich_ban_Social.xlsx
+++ b/SunLife_Kich_ban_Social.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -493,6 +493,7 @@
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="28" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -510,7 +511,7 @@
     <row r="2" ht="75" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Dữ liệu lấy từ sunlife.com.vn (xem cột Nguồn).  VÀNG = cần KH bổ sung (chưa có dữ liệu)  |  CAM NHẠT = cần KH xác nhận.  Tổng hợp câu hỏi ở tab 'Câu hỏi cho KH'.</t>
+          <t>Dữ liệu lấy từ sunlife.com.vn (xem cột Link nguồn).  VÀNG = cần KH bổ sung (chưa có dữ liệu)  |  CAM NHẠT = cần KH xác nhận.  Tổng hợp câu hỏi ở tab 'Câu hỏi cho KH'.</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -543,14 +544,14 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
+          <t>Link nguồn</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
           <t>Câu hỏi cho khách hàng</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Nguồn</t>
-        </is>
-      </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Thông tin tài khoản</t>
@@ -567,6 +568,11 @@
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Link nguồn</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>Câu hỏi cho khách hàng</t>
         </is>
@@ -591,12 +597,12 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
         </is>
       </c>
+      <c r="F4" s="6" t="inlineStr"/>
       <c r="H4" s="7" t="inlineStr">
         <is>
           <t>Username</t>
@@ -612,7 +618,12 @@
           <t>Đề xuất (trùng tên Facebook/Youtube chính thức)</t>
         </is>
       </c>
-      <c r="K4" s="7" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/SunLifeVietnam</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
         <is>
           <t>Đồng ý dùng 'sunlifevietnam' làm username? Nếu bị trùng, dùng phương án nào (VD: sunlifevn, sunlife.vietnam)?</t>
         </is>
@@ -637,12 +648,12 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
         </is>
       </c>
+      <c r="F5" s="6" t="inlineStr"/>
       <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Tên hiển thị</t>
@@ -658,7 +669,12 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
         <is>
           <t>Xác nhận tên hiển thị 'Sun Life Việt Nam'.</t>
         </is>
@@ -683,14 +699,14 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>Lĩnh vực public trên social ghi 'Bảo hiểm nhân thọ' là đủ, hay cần ghi chi tiết hơn (VD: Bảo hiểm nhân thọ &amp; Hưu trí)?</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -704,7 +720,12 @@
           <t>Team SEO cấp email riêng</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr"/>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>Nội bộ SEO</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr"/>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="6" t="n">
@@ -725,14 +746,14 @@
           <t>ok – Địa chỉ trụ sở theo trang Liên hệ. Chi nhánh: Hà Nội – Tầng 22 Tòa nhà Capital Place, 29 Liễu Giai, Phường Ngọc Hà, Hà Nội; Đà Nẵng – Tòa nhà Nexus, Số 75-77-79 Xô Viết Nghệ Tĩnh, Phường Cẩm Lệ, TP. Đà Nẵng</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>Xác nhận dùng địa chỉ trụ sở mới (phường Sài Gòn, TP.HCM) cho mọi tài khoản social? Có cần thêm địa chỉ chi nhánh Hà Nội, Đà Nẵng không?</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -746,7 +767,12 @@
           <t>Team SEO đặt</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>Nội bộ SEO</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="6" t="inlineStr"/>
@@ -762,15 +788,19 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Mã bưu chính chung TP.HCM (không lấy từ website)</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
+          <t>Mã bưu chính chung TP.HCM</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Không có trên website</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>Zipcode dùng 700000 (mã chung TP.HCM) được không, hay doanh nghiệp có mã bưu chính riêng?</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr"/>
       <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Zip code</t>
@@ -783,10 +813,15 @@
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="K8" s="6" t="inlineStr"/>
+          <t>Mã bưu chính chung TP.HCM</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>Không có trên website</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr"/>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="6" t="n">
@@ -808,14 +843,14 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>Số chính public trên social là hotline 1800 1786? Có được public thêm số (028) 6298 5888 không?</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -826,6 +861,7 @@
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -846,16 +882,16 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Email Dichvu.Khachhang@sunlife.com có được public trên social không, hay dùng email khác?</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
-        </is>
-      </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Giới tính</t>
@@ -872,6 +908,7 @@
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -894,18 +931,18 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Có mốc lịch sử nào khác muốn bổ sung? Có được public thông tin vốn điều lệ 18.909 tỷ đồng không?</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/
 https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2016/tap-doan-tai-chinh-sun-life-hoan-tat-thuong-vu-chuyen-nhuong-25-co-phan-con-lai-tu-cong-ty-pvi-sun-life
 https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2026/sun-life-viet-nam-tang-von-dieu-le-len-18909-ty-dong/</t>
         </is>
       </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Có mốc lịch sử nào khác muốn bổ sung? Có được public thông tin vốn điều lệ 18.909 tỷ đồng không?</t>
+        </is>
+      </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
           <t>Ngày sinh/Ngày thành lập</t>
@@ -921,7 +958,12 @@
           <t>Website chỉ ghi năm 2013 – cần KH cung cấp ngày cụ thể</t>
         </is>
       </c>
-      <c r="K11" s="8" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
+        </is>
+      </c>
+      <c r="L11" s="8" t="inlineStr">
         <is>
           <t>Ngày thành lập chính thức (dd/mm/yyyy) là ngày nào?</t>
         </is>
@@ -947,17 +989,17 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>Giờ hoạt động public trên social dùng giờ tổng đài (8:00–18:00, T2–T6) hay giờ Trung tâm Dịch vụ Khách hàng (có sáng T7)?</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/tong-dai-cham-soc-khach-hang/
 https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/mang-luoi-trung-tam-dich-vu-khach-hang/</t>
         </is>
       </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Giờ hoạt động public trên social dùng giờ tổng đài (8:00–18:00, T2–T6) hay giờ Trung tâm Dịch vụ Khách hàng (có sáng T7)?</t>
+        </is>
+      </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
           <t>Website</t>
@@ -973,7 +1015,12 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="K12" s="6" t="inlineStr"/>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr"/>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -995,17 +1042,17 @@
           <t>Cần KH xác nhận danh sách giải thưởng/chứng nhận muốn đưa lên social</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Gửi danh sách giải thưởng/chứng nhận chính thức muốn public (tên giải, năm, đơn vị trao).</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/cac-giai-thuong/
 https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2023/noi-lam-viec-tot-2023/</t>
         </is>
       </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Gửi danh sách giải thưởng/chứng nhận chính thức muốn public (tên giải, năm, đơn vị trao).</t>
+        </is>
+      </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
           <t>Logo - Avatar</t>
@@ -1017,7 +1064,8 @@
           <t>Cần KH cung cấp file logo gốc</t>
         </is>
       </c>
-      <c r="K13" s="8" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr"/>
+      <c r="L13" s="8" t="inlineStr">
         <is>
           <t>Gửi file logo gốc (PNG nền trong, ≥1000px, có bản vuông cho avatar).</t>
         </is>
@@ -1038,12 +1086,16 @@
           <t>Cần KH cung cấp</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Không có trên website</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>Có khách hàng (doanh nghiệp) tiêu biểu nào được phép công bố trên social không? Nếu có, gửi danh sách.</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr"/>
       <c r="H14" s="8" t="inlineStr">
         <is>
           <t>Banner</t>
@@ -1055,7 +1107,8 @@
           <t>Cần KH cung cấp file banner</t>
         </is>
       </c>
-      <c r="K14" s="8" t="inlineStr">
+      <c r="K14" s="6" t="inlineStr"/>
+      <c r="L14" s="8" t="inlineStr">
         <is>
           <t>Gửi banner/ảnh bìa (gợi ý 1500x500px) hoặc đồng ý cho dùng ảnh bìa Facebook hiện tại.</t>
         </is>
@@ -1080,14 +1133,14 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2020/sun-life-viet-nam-va-acb-thoa-thuan-doc-quyen-phan-phoi-bao-hiem-nhan-tho/</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>Ngoài ACB, còn đối tác nào (ngân hàng, đối tác chiến lược) muốn đưa lên social không?</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2020/sun-life-viet-nam-va-acb-thoa-thuan-doc-quyen-phan-phoi-bao-hiem-nhan-tho/</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -1108,7 +1161,12 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="K15" s="6" t="inlineStr"/>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/dich-vu-khach-hang/chuong-trinh-khuyen-mai/2025/</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -1129,7 +1187,11 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr"/>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/</t>
+        </is>
+      </c>
       <c r="F16" s="6" t="inlineStr"/>
     </row>
     <row r="17" ht="60" customHeight="1">
@@ -1154,14 +1216,14 @@
           <t>ok – Chưa có link Zalo OA/LinkedIn/TikTok, cần KH cung cấp</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/dich-vu-khach-hang/chuong-trinh-khuyen-mai/2025/</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>Gửi link Zalo OA, LinkedIn, TikTok (nếu có) và xác nhận link Facebook/Youtube/Instagram chính thức.</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/dich-vu-khach-hang/chuong-trinh-khuyen-mai/2025/</t>
         </is>
       </c>
     </row>
@@ -1184,14 +1246,14 @@
           <t>Thông điệp chiến dịch thương hiệu trên website – cần KH xác nhận slogan chính thức</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2024/lac-quan-tai-chinh/</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>Slogan chính thức của Sun Life Việt Nam là gì? Có dùng thông điệp 'Tài chính cho mình. Lạc quan do mình' làm slogan được không?</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2024/lac-quan-tai-chinh/</t>
         </is>
       </c>
     </row>
@@ -1222,14 +1284,14 @@
           <t>Ghép nguyên văn các câu giới thiệu trên website; hashtag do team SEO đề xuất</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>Duyệt nội dung Bio ngắn (câu giới thiệu lấy nguyên văn từ website). Thương hiệu có bộ hashtag chính thức không?</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
         </is>
       </c>
     </row>
@@ -1260,14 +1322,14 @@
           <t>Ghép nguyên văn các câu giới thiệu trên website; hashtag do team SEO đề xuất</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>Duyệt nội dung Bio trung bình – có câu nào cần sửa/thêm không?</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
         </is>
       </c>
     </row>
@@ -1300,15 +1362,15 @@
           <t>Ghép nguyên văn các câu giới thiệu trên website; hashtag do team SEO đề xuất</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>Duyệt nội dung Bio dài – có muốn bổ sung sản phẩm/thông điệp chủ lực nào không?</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/
 https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Duyệt nội dung Bio dài – có muốn bổ sung sản phẩm/thông điệp chủ lực nào không?</t>
         </is>
       </c>
     </row>
@@ -1324,15 +1386,19 @@
       <c r="C22" s="6" t="inlineStr"/>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Cần KH cung cấp – không tìm thấy mục Giá trị cốt lõi của công ty trên website</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
+          <t>Cần KH cung cấp</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Không có trên website</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>Gửi nội dung Giá trị cốt lõi chính thức của Sun Life Việt Nam.</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr"/>
     </row>
     <row r="23" ht="45" customHeight="1">
       <c r="A23" s="6" t="n">
@@ -1345,22 +1411,22 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Mục đích: Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn.</t>
+          <t>Mục đích (trên website): Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn.</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Website chỉ nêu Mục đích; Tầm nhìn – Sứ mệnh chi tiết cần kh cung cấp</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
+          <t>Website KHÔNG có mục Tầm nhìn/Sứ mệnh – chỉ có câu Mục đích trong trang Giới thiệu công ty. Tầm nhìn – Sứ mệnh cần KH cung cấp</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Gửi nội dung Tầm nhìn, Sứ mệnh chính thức (hay chỉ dùng Mục đích của Tập đoàn như trên website)?</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
         </is>
       </c>
     </row>
@@ -1397,22 +1463,22 @@
           <t>Theo trang Hội đồng Thành viên &amp; Ban Điều hành – có thể chưa đủ toàn bộ thành viên, nên mở link kiểm tra</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>Xác nhận danh sách Hội đồng Thành viên &amp; Ban Điều hành mới nhất. Có được public tên lãnh đạo trên social không?</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/hoi-dong-thanh-vien/
 https://www.sunlife.com.vn/vn/ve-chung-toi/hoi-dong-thanh-vien/ban-dieu-hanh/</t>
         </is>
       </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Xác nhận danh sách Hội đồng Thành viên &amp; Ban Điều hành mới nhất. Có được public tên lãnh đạo trên social không?</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="H2:K2"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="H2:L2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1663,7 +1729,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Mục đích: Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn.</t>
+          <t>Mục đích (trên website): Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn.</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Attach clickable source links for all proposed content; add references tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR1qVnPwb7hxUbF4akMpvt
</commit_message>
<xml_diff>
--- a/SunLife_Kich_ban_Social.xlsx
+++ b/SunLife_Kich_ban_Social.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Kịch bản Social" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Câu hỏi cho KH" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Nguồn tham khảo" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,6 +36,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
     <font>
       <b val="1"/>
@@ -90,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -106,14 +111,24 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -597,13 +612,13 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>Username</t>
         </is>
@@ -613,17 +628,18 @@
           <t>sunlifevietnam</t>
         </is>
       </c>
-      <c r="J4" s="7" t="inlineStr">
-        <is>
-          <t>Đề xuất (trùng tên Facebook/Youtube chính thức)</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/SunLifeVietnam</t>
-        </is>
-      </c>
-      <c r="L4" s="7" t="inlineStr">
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>Đề xuất theo tên kênh chính thức facebook.com/SunLifeVietnam, youtube.com/c/SunLifeVietnam</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/SunLifeVietnam
+https://www.youtube.com/c/SunLifeVietnam</t>
+        </is>
+      </c>
+      <c r="L4" s="8" t="inlineStr">
         <is>
           <t>Đồng ý dùng 'sunlifevietnam' làm username? Nếu bị trùng, dùng phương án nào (VD: sunlifevn, sunlife.vietnam)?</t>
         </is>
@@ -648,13 +664,13 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>Tên hiển thị</t>
         </is>
@@ -664,17 +680,17 @@
           <t>Sun Life Việt Nam</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr">
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Xác nhận tên hiển thị 'Sun Life Việt Nam'.</t>
         </is>
@@ -684,7 +700,7 @@
       <c r="A6" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Lĩnh vực kinh doanh</t>
         </is>
@@ -694,17 +710,17 @@
           <t>Bảo hiểm nhân thọ</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Lĩnh vực public trên social ghi 'Bảo hiểm nhân thọ' là đủ, hay cần ghi chi tiết hơn (VD: Bảo hiểm nhân thọ &amp; Hưu trí)?</t>
         </is>
@@ -731,7 +747,7 @@
       <c r="A7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Địa chỉ</t>
         </is>
@@ -741,17 +757,17 @@
           <t>Tầng 29, Tòa nhà Vietcombank Tower, số 05 Công trường Mê Linh, phường Sài Gòn, Thành phố Hồ Chí Minh</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>ok – Địa chỉ trụ sở theo trang Liên hệ. Chi nhánh: Hà Nội – Tầng 22 Tòa nhà Capital Place, 29 Liễu Giai, Phường Ngọc Hà, Hà Nội; Đà Nẵng – Tòa nhà Nexus, Số 75-77-79 Xô Viết Nghệ Tĩnh, Phường Cẩm Lệ, TP. Đà Nẵng</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Xác nhận dùng địa chỉ trụ sở mới (phường Sài Gòn, TP.HCM) cho mọi tài khoản social? Có cần thêm địa chỉ chi nhánh Hà Nội, Đà Nẵng không?</t>
         </is>
@@ -776,7 +792,7 @@
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="6" t="inlineStr"/>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Zipcode</t>
         </is>
@@ -786,17 +802,18 @@
           <t>700000</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>Mã bưu chính chung TP.HCM</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Không có trên website</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Mã bưu chính chung TP.HCM | Nguồn: Mã bưu chính chung TP.HCM (nguồn ngoài website KH)</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Postal_codes_in_Vietnam
+https://ghtk.vn/blog/ma-zip-thanh-pho-ho-chi-minh/</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Zipcode dùng 700000 (mã chung TP.HCM) được không, hay doanh nghiệp có mã bưu chính riêng?</t>
         </is>
@@ -813,12 +830,13 @@
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Mã bưu chính chung TP.HCM</t>
-        </is>
-      </c>
-      <c r="K8" s="6" t="inlineStr">
-        <is>
-          <t>Không có trên website</t>
+          <t>Mã bưu chính chung TP.HCM (nguồn ngoài website KH)</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Postal_codes_in_Vietnam
+https://ghtk.vn/blog/ma-zip-thanh-pho-ho-chi-minh/</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr"/>
@@ -827,7 +845,7 @@
       <c r="A9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Số điện thoại</t>
         </is>
@@ -838,17 +856,18 @@
 Điện thoại: (028) 6298 5888</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/
+https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/tong-dai-cham-soc-khach-hang/</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Số chính public trên social là hotline 1800 1786? Có được public thêm số (028) 6298 5888 không?</t>
         </is>
@@ -867,7 +886,7 @@
       <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
@@ -877,17 +896,17 @@
           <t>Dichvu.Khachhang@sunlife.com</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>Email Dichvu.Khachhang@sunlife.com có được public trên social không, hay dùng email khác?</t>
         </is>
@@ -914,7 +933,7 @@
       <c r="A11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Lịch sử hoạt động</t>
         </is>
@@ -926,24 +945,24 @@
 - 2026: Được Bộ Tài chính chấp thuận tăng vốn điều lệ lên 18.909 tỷ đồng</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/
 https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2016/tap-doan-tai-chinh-sun-life-hoan-tat-thuong-vu-chuyen-nhuong-25-co-phan-con-lai-tu-cong-ty-pvi-sun-life
 https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2026/sun-life-viet-nam-tang-von-dieu-le-len-18909-ty-dong/</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>Có mốc lịch sử nào khác muốn bổ sung? Có được public thông tin vốn điều lệ 18.909 tỷ đồng không?</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>Ngày sinh/Ngày thành lập</t>
         </is>
@@ -953,17 +972,18 @@
           <t>2013</t>
         </is>
       </c>
-      <c r="J11" s="8" t="inlineStr">
+      <c r="J11" s="9" t="inlineStr">
         <is>
           <t>Website chỉ ghi năm 2013 – cần KH cung cấp ngày cụ thể</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
-        </is>
-      </c>
-      <c r="L11" s="8" t="inlineStr">
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/
+https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2016/tap-doan-tai-chinh-sun-life-hoan-tat-thuong-vu-chuyen-nhuong-25-co-phan-con-lai-tu-cong-ty-pvi-sun-life</t>
+        </is>
+      </c>
+      <c r="L11" s="9" t="inlineStr">
         <is>
           <t>Ngày thành lập chính thức (dd/mm/yyyy) là ngày nào?</t>
         </is>
@@ -973,7 +993,7 @@
       <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Thời gian hoạt động</t>
         </is>
@@ -984,18 +1004,18 @@
 Trung tâm Dịch vụ Khách hàng: Thứ 2 - Thứ 6: 8:30 - 12:00 và 13:00 - 17:30; Thứ 7: 8:30 - 12:00</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/tong-dai-cham-soc-khach-hang/
 https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/mang-luoi-trung-tam-dich-vu-khach-hang/</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>Giờ hoạt động public trên social dùng giờ tổng đài (8:00–18:00, T2–T6) hay giờ Trung tâm Dịch vụ Khách hàng (có sáng T7)?</t>
         </is>
@@ -1015,7 +1035,7 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="K12" s="6" t="inlineStr">
+      <c r="K12" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/</t>
         </is>
@@ -1026,7 +1046,7 @@
       <c r="A13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Bằng cấp, giải thưởng, chứng nhận...</t>
         </is>
@@ -1037,35 +1057,39 @@
 - Great Place To Work® 2022–2025</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>Cần KH xác nhận danh sách giải thưởng/chứng nhận muốn đưa lên social</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/cac-giai-thuong/
 https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2023/noi-lam-viec-tot-2023/</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>Gửi danh sách giải thưởng/chứng nhận chính thức muốn public (tên giải, năm, đơn vị trao).</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>Logo - Avatar</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr"/>
-      <c r="J13" s="8" t="inlineStr">
-        <is>
-          <t>Cần KH cung cấp file logo gốc</t>
-        </is>
-      </c>
-      <c r="K13" s="6" t="inlineStr"/>
-      <c r="L13" s="8" t="inlineStr">
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>Logo hiện dùng trên Facebook chính thức – cần KH gửi file gốc</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/SunLifeVietnam</t>
+        </is>
+      </c>
+      <c r="L13" s="9" t="inlineStr">
         <is>
           <t>Gửi file logo gốc (PNG nền trong, ≥1000px, có bản vuông cho avatar).</t>
         </is>
@@ -1075,13 +1099,13 @@
       <c r="A14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Khách hàng nổi bật (nếu có)</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr"/>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>Cần KH cung cấp</t>
         </is>
@@ -1091,24 +1115,28 @@
           <t>Không có trên website</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>Có khách hàng (doanh nghiệp) tiêu biểu nào được phép công bố trên social không? Nếu có, gửi danh sách.</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
+      <c r="H14" s="9" t="inlineStr">
         <is>
           <t>Banner</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr"/>
-      <c r="J14" s="8" t="inlineStr">
-        <is>
-          <t>Cần KH cung cấp file banner</t>
-        </is>
-      </c>
-      <c r="K14" s="6" t="inlineStr"/>
-      <c r="L14" s="8" t="inlineStr">
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t>Ảnh bìa hiện dùng trên Facebook chính thức – cần KH gửi file gốc</t>
+        </is>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/SunLifeVietnam</t>
+        </is>
+      </c>
+      <c r="L14" s="9" t="inlineStr">
         <is>
           <t>Gửi banner/ảnh bìa (gợi ý 1500x500px) hoặc đồng ý cho dùng ảnh bìa Facebook hiện tại.</t>
         </is>
@@ -1118,7 +1146,7 @@
       <c r="A15" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Đối tác tiêu biểu (nếu có)</t>
         </is>
@@ -1128,17 +1156,17 @@
           <t>Ngân hàng TMCP Á Châu (ACB) – thỏa thuận hợp tác độc quyền phân phối sản phẩm bảo hiểm nhân thọ kéo dài 15 năm (công bố năm 2020)</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2020/sun-life-viet-nam-va-acb-thoa-thuan-doc-quyen-phan-phoi-bao-hiem-nhan-tho/</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Ngoài ACB, còn đối tác nào (ngân hàng, đối tác chiến lược) muốn đưa lên social không?</t>
         </is>
@@ -1161,9 +1189,12 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="K15" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/dich-vu-khach-hang/chuong-trinh-khuyen-mai/2025/</t>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/SunLifeVietnam
+https://www.youtube.com/c/SunLifeVietnam
+https://www.instagram.com/sunlifevn/
+https://www.sunlife.com.vn/vn/dich-vu-khach-hang/chuong-trinh-khuyen-mai/2025/</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr"/>
@@ -1187,7 +1218,7 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/</t>
         </is>
@@ -1198,7 +1229,7 @@
       <c r="A17" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Social chính</t>
         </is>
@@ -1211,17 +1242,20 @@
 Zalo Official Account: Sun Life Việt Nam</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>ok – Chưa có link Zalo OA/LinkedIn/TikTok, cần KH cung cấp</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/dich-vu-khach-hang/chuong-trinh-khuyen-mai/2025/</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/SunLifeVietnam
+https://www.youtube.com/c/SunLifeVietnam
+https://www.instagram.com/sunlifevn/
+https://www.sunlife.com.vn/vn/dich-vu-khach-hang/chuong-trinh-khuyen-mai/2025/</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>Gửi link Zalo OA, LinkedIn, TikTok (nếu có) và xác nhận link Facebook/Youtube/Instagram chính thức.</t>
         </is>
@@ -1231,7 +1265,7 @@
       <c r="A18" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Slogan</t>
         </is>
@@ -1241,17 +1275,17 @@
           <t>Tài chính cho mình. Lạc quan do mình</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Thông điệp chiến dịch thương hiệu trên website – cần KH xác nhận slogan chính thức</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2024/lac-quan-tai-chinh/</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>Slogan chính thức của Sun Life Việt Nam là gì? Có dùng thông điệp 'Tài chính cho mình. Lạc quan do mình' làm slogan được không?</t>
         </is>
@@ -1261,7 +1295,7 @@
       <c r="A19" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Bio ngắn</t>
         </is>
@@ -1279,17 +1313,21 @@
 #SunLifeVietnam #SunLife #BaoHiemNhanTho #BaoHiemHuuTri</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>Ghép nguyên văn các câu giới thiệu trên website; hashtag do team SEO đề xuất</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Ghép nguyên văn các câu giới thiệu trên website; hashtag do team SEO đề xuất | Nguồn: Câu giới thiệu: Về chúng tôi; liên hệ: Liên hệ; hashtag: team SEO đề xuất (không có nguồn)</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/
+https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/
+https://www.facebook.com/SunLifeVietnam
+https://www.youtube.com/c/SunLifeVietnam
+https://www.instagram.com/sunlifevn/</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>Duyệt nội dung Bio ngắn (câu giới thiệu lấy nguyên văn từ website). Thương hiệu có bộ hashtag chính thức không?</t>
         </is>
@@ -1299,7 +1337,7 @@
       <c r="A20" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Bio trung bình</t>
         </is>
@@ -1317,17 +1355,22 @@
 #SunLifeVietnam #SunLife #BaoHiemNhanTho #BaoHiemHuuTri</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>Ghép nguyên văn các câu giới thiệu trên website; hashtag do team SEO đề xuất</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Ghép nguyên văn các câu giới thiệu trên website; hashtag do team SEO đề xuất | Nguồn: Câu giới thiệu: Về chúng tôi; câu mục đích: Giới thiệu công ty; hashtag: team SEO đề xuất</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/
+https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/
+https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/
+https://www.facebook.com/SunLifeVietnam
+https://www.youtube.com/c/SunLifeVietnam
+https://www.instagram.com/sunlifevn/</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>Duyệt nội dung Bio trung bình – có câu nào cần sửa/thêm không?</t>
         </is>
@@ -1337,7 +1380,7 @@
       <c r="A21" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Bio dài + Có link social</t>
         </is>
@@ -1357,18 +1400,22 @@
 #SunLifeVietnam #SunLife #BaoHiemNhanTho #BaoHiemHuuTri</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>Ghép nguyên văn các câu giới thiệu trên website; hashtag do team SEO đề xuất</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Ghép nguyên văn các câu giới thiệu trên website; hashtag do team SEO đề xuất | Nguồn: Câu giới thiệu: Về chúng tôi; lịch sử, mục đích, tiên phong hưu trí: Giới thiệu công ty; hashtag: team SEO đề xuất</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/
-https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
+https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/
+https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/
+https://www.facebook.com/SunLifeVietnam
+https://www.youtube.com/c/SunLifeVietnam
+https://www.instagram.com/sunlifevn/</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>Duyệt nội dung Bio dài – có muốn bổ sung sản phẩm/thông điệp chủ lực nào không?</t>
         </is>
@@ -1378,13 +1425,13 @@
       <c r="A22" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Giá trị cốt lõi</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr"/>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Cần KH cung cấp</t>
         </is>
@@ -1394,7 +1441,7 @@
           <t>Không có trên website</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Gửi nội dung Giá trị cốt lõi chính thức của Sun Life Việt Nam.</t>
         </is>
@@ -1404,7 +1451,7 @@
       <c r="A23" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Tầm nhìn - Sứ mệnh</t>
         </is>
@@ -1414,17 +1461,17 @@
           <t>Mục đích (trên website): Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn.</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>Website KHÔNG có mục Tầm nhìn/Sứ mệnh – chỉ có câu Mục đích trong trang Giới thiệu công ty. Tầm nhìn – Sứ mệnh cần KH cung cấp</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>Gửi nội dung Tầm nhìn, Sứ mệnh chính thức (hay chỉ dùng Mục đích của Tập đoàn như trên website)?</t>
         </is>
@@ -1434,7 +1481,7 @@
       <c r="A24" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>Đội ngũ nhân sự</t>
         </is>
@@ -1458,18 +1505,18 @@
 - Phó TGĐ Sáng kiến Chiến lược: Ông Phạm Công Kháng</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>Theo trang Hội đồng Thành viên &amp; Ban Điều hành – có thể chưa đủ toàn bộ thành viên, nên mở link kiểm tra</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>https://www.sunlife.com.vn/vn/ve-chung-toi/hoi-dong-thanh-vien/
 https://www.sunlife.com.vn/vn/ve-chung-toi/hoi-dong-thanh-vien/ban-dieu-hanh/</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>Xác nhận danh sách Hội đồng Thành viên &amp; Ban Điều hành mới nhất. Có được public tên lãnh đạo trên social không?</t>
         </is>
@@ -1481,6 +1528,35 @@
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId27"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1504,14 +1580,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>DANH SÁCH CÂU HỎI GỬI KHÁCH HÀNG – SUN LIFE VIỆT NAM</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>KH vui lòng điền vào cột 'Câu trả lời của KH'. VÀNG = cần bổ sung, CAM NHẠT = cần xác nhận.</t>
         </is>
@@ -1563,7 +1639,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Bằng cấp, giải thưởng, chứng nhận...</t>
         </is>
@@ -1574,12 +1650,12 @@
 - Great Place To Work® 2022–2025</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>Gửi danh sách giải thưởng/chứng nhận chính thức muốn public (tên giải, năm, đơn vị trao).</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Cần bổ sung</t>
         </is>
@@ -1595,7 +1671,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Khách hàng nổi bật (nếu có)</t>
         </is>
@@ -1605,12 +1681,12 @@
           <t>(trống)</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>Có khách hàng (doanh nghiệp) tiêu biểu nào được phép công bố trên social không? Nếu có, gửi danh sách.</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>Cần bổ sung</t>
         </is>
@@ -1626,7 +1702,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Social chính</t>
         </is>
@@ -1639,12 +1715,12 @@
 Zalo Official Account: Sun Life Việt Nam</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Gửi link Zalo OA, LinkedIn, TikTok (nếu có) và xác nhận link Facebook/Youtube/Instagram chính thức.</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>Cần bổ sung</t>
         </is>
@@ -1660,7 +1736,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Slogan</t>
         </is>
@@ -1670,12 +1746,12 @@
           <t>Tài chính cho mình. Lạc quan do mình</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>Slogan chính thức của Sun Life Việt Nam là gì? Có dùng thông điệp 'Tài chính cho mình. Lạc quan do mình' làm slogan được không?</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>Cần bổ sung</t>
         </is>
@@ -1691,7 +1767,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Giá trị cốt lõi</t>
         </is>
@@ -1701,12 +1777,12 @@
           <t>(trống)</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>Gửi nội dung Giá trị cốt lõi chính thức của Sun Life Việt Nam.</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>Cần bổ sung</t>
         </is>
@@ -1722,7 +1798,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Tầm nhìn - Sứ mệnh</t>
         </is>
@@ -1732,12 +1808,12 @@
           <t>Mục đích (trên website): Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng cuộc sống khoẻ mạnh hơn.</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>Gửi nội dung Tầm nhìn, Sứ mệnh chính thức (hay chỉ dùng Mục đích của Tập đoàn như trên website)?</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Cần bổ sung</t>
         </is>
@@ -1753,7 +1829,7 @@
           <t>Tạo tài khoản</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Ngày sinh/Ngày thành lập</t>
         </is>
@@ -1763,12 +1839,12 @@
           <t>2013</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>Ngày thành lập chính thức (dd/mm/yyyy) là ngày nào?</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>Cần bổ sung</t>
         </is>
@@ -1784,7 +1860,7 @@
           <t>Tạo tài khoản</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>Logo - Avatar</t>
         </is>
@@ -1794,12 +1870,12 @@
           <t>(trống)</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>Gửi file logo gốc (PNG nền trong, ≥1000px, có bản vuông cho avatar).</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>Cần bổ sung</t>
         </is>
@@ -1815,7 +1891,7 @@
           <t>Tạo tài khoản</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Banner</t>
         </is>
@@ -1825,12 +1901,12 @@
           <t>(trống)</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>Gửi banner/ảnh bìa (gợi ý 1500x500px) hoặc đồng ý cho dùng ảnh bìa Facebook hiện tại.</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>Cần bổ sung</t>
         </is>
@@ -1846,7 +1922,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Lĩnh vực kinh doanh</t>
         </is>
@@ -1856,12 +1932,12 @@
           <t>Bảo hiểm nhân thọ</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>Lĩnh vực public trên social ghi 'Bảo hiểm nhân thọ' là đủ, hay cần ghi chi tiết hơn (VD: Bảo hiểm nhân thọ &amp; Hưu trí)?</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>Cần xác nhận</t>
         </is>
@@ -1877,7 +1953,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Địa chỉ</t>
         </is>
@@ -1887,12 +1963,12 @@
           <t>Tầng 29, Tòa nhà Vietcombank Tower, số 05 Công trường Mê Linh, phường Sài Gòn, Thành phố Hồ Chí Minh</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Xác nhận dùng địa chỉ trụ sở mới (phường Sài Gòn, TP.HCM) cho mọi tài khoản social? Có cần thêm địa chỉ chi nhánh Hà Nội, Đà Nẵng không?</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>Cần xác nhận</t>
         </is>
@@ -1908,7 +1984,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Zipcode</t>
         </is>
@@ -1918,12 +1994,12 @@
           <t>700000</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Zipcode dùng 700000 (mã chung TP.HCM) được không, hay doanh nghiệp có mã bưu chính riêng?</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Cần xác nhận</t>
         </is>
@@ -1939,7 +2015,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Số điện thoại</t>
         </is>
@@ -1950,12 +2026,12 @@
 Điện thoại: (028) 6298 5888</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>Số chính public trên social là hotline 1800 1786? Có được public thêm số (028) 6298 5888 không?</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>Cần xác nhận</t>
         </is>
@@ -1971,7 +2047,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
@@ -1981,12 +2057,12 @@
           <t>Dichvu.Khachhang@sunlife.com</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Email Dichvu.Khachhang@sunlife.com có được public trên social không, hay dùng email khác?</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>Cần xác nhận</t>
         </is>
@@ -2002,7 +2078,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>Lịch sử hoạt động</t>
         </is>
@@ -2014,12 +2090,12 @@
 - 2026: Được Bộ Tài chính chấp thuận tăng vốn điều…</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>Có mốc lịch sử nào khác muốn bổ sung? Có được public thông tin vốn điều lệ 18.909 tỷ đồng không?</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>Cần xác nhận</t>
         </is>
@@ -2035,7 +2111,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Thời gian hoạt động</t>
         </is>
@@ -2046,12 +2122,12 @@
 Trung tâm Dịch vụ Khách hàng: Thứ 2 - Thứ 6: 8:30 - 12:00 và 13:00 - 17:30; Thứ 7: 8:30 - 12:00</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>Giờ hoạt động public trên social dùng giờ tổng đài (8:00–18:00, T2–T6) hay giờ Trung tâm Dịch vụ Khách hàng (có sáng T7)?</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>Cần xác nhận</t>
         </is>
@@ -2067,7 +2143,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>Đối tác tiêu biểu (nếu có)</t>
         </is>
@@ -2077,12 +2153,12 @@
           <t>Ngân hàng TMCP Á Châu (ACB) – thỏa thuận hợp tác độc quyền phân phối sản phẩm bảo hiểm nhân thọ kéo dài 15 năm (công bố năm 2020)</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>Ngoài ACB, còn đối tác nào (ngân hàng, đối tác chiến lược) muốn đưa lên social không?</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>Cần xác nhận</t>
         </is>
@@ -2098,7 +2174,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Bio ngắn</t>
         </is>
@@ -2109,12 +2185,12 @@
 Địa chỉ: Tầng 29, Tòa nhà Vietcombank Tower, số 05 Công trường Mê Linh, phường Sài Gòn, Thành phố Hồ C…</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Duyệt nội dung Bio ngắn (câu giới thiệu lấy nguyên văn từ website). Thương hiệu có bộ hashtag chính thức không?</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>Cần xác nhận</t>
         </is>
@@ -2130,7 +2206,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>Bio trung bình</t>
         </is>
@@ -2140,12 +2216,12 @@
           <t>Sun Life Việt Nam là thành viên của tập đoàn Sun Life (trụ sở tại Canada) – Tổ chức dịch vụ tài chính quốc tế hàng đầu với kinh nghiệm hoạt động trên 157 năm có mặt ở nhiều quốc gia trên thế giới. Sun Life Việt Nam hướng đến mục đích giúp Khách hàng đạt được an toàn tài chính trọn đời và tận hưởng c…</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>Duyệt nội dung Bio trung bình – có câu nào cần sửa/thêm không?</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>Cần xác nhận</t>
         </is>
@@ -2161,7 +2237,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Bio dài + Có link social</t>
         </is>
@@ -2172,12 +2248,12 @@
 Năm 2013, Sun Life đặt chân đến thị trường Việt Nam thông qua liên doanh Bảo hiểm Nhân thọ PVI Sun Lif…</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>Duyệt nội dung Bio dài – có muốn bổ sung sản phẩm/thông điệp chủ lực nào không?</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Cần xác nhận</t>
         </is>
@@ -2193,7 +2269,7 @@
           <t>Thông tin public</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>Đội ngũ nhân sự</t>
         </is>
@@ -2211,12 +2287,12 @@
 - Phó TGĐ Kênh Đại lý: Ông Budi D…</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>Xác nhận danh sách Hội đồng Thành viên &amp; Ban Điều hành mới nhất. Có được public tên lãnh đạo trên social không?</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>Cần xác nhận</t>
         </is>
@@ -2232,7 +2308,7 @@
           <t>Tạo tài khoản</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>Username</t>
         </is>
@@ -2242,12 +2318,12 @@
           <t>sunlifevietnam</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>Đồng ý dùng 'sunlifevietnam' làm username? Nếu bị trùng, dùng phương án nào (VD: sunlifevn, sunlife.vietnam)?</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>Cần xác nhận</t>
         </is>
@@ -2263,7 +2339,7 @@
           <t>Tạo tài khoản</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>Tên hiển thị</t>
         </is>
@@ -2273,12 +2349,12 @@
           <t>Sun Life Việt Nam</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
         <is>
           <t>Xác nhận tên hiển thị 'Sun Life Việt Nam'.</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="F26" s="8" t="inlineStr">
         <is>
           <t>Cần xác nhận</t>
         </is>
@@ -2319,4 +2395,454 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>Trang</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>Thông tin đã lấy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>Về chúng tôi</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>Câu giới thiệu dùng trong 3 bio; tên thương hiệu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Giới thiệu công ty</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/gioi-thieu-cong-ty/</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Lĩnh vực; lịch sử 2013/2016; câu Mục đích; tiên phong hưu trí</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Liên hệ</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Tên đầy đủ; địa chỉ trụ sở &amp; chi nhánh; điện thoại; email</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Tổng đài Chăm sóc Khách hàng</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/tong-dai-cham-soc-khach-hang/</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Hotline 1800 1786; giờ hỗ trợ của tổng đài</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Mạng lưới Trung tâm Dịch vụ Khách hàng</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/lien-he/mang-luoi-trung-tam-dich-vu-khach-hang/</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Giờ làm việc Trung tâm DVKH</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Tin 2016 – hoàn tất chuyển nhượng 25% PVI Sun Life</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2016/tap-doan-tai-chinh-sun-life-hoan-tat-thuong-vu-chuyen-nhuong-25-co-phan-con-lai-tu-cong-ty-pvi-sun-life</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Mốc 11/2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Tin 2026 – tăng vốn điều lệ 18.909 tỷ đồng</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2026/sun-life-viet-nam-tang-von-dieu-le-len-18909-ty-dong/</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Mốc 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Các giải thưởng</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/cac-giai-thuong/</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Giải Dịch vụ khách hàng tốt nhất 2024; Great Place To Work®</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Tin 2023 – Nơi làm việc xuất sắc</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2023/noi-lam-viec-tot-2023/</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Great Place To Work® 2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Tin 2020 – hợp tác độc quyền với ACB</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2020/sun-life-viet-nam-va-acb-thoa-thuan-doc-quyen-phan-phoi-bao-hiem-nhan-tho/</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Đối tác tiêu biểu</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Tin 2024 – Tài chính cho mình, lạc quan do mình</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/tin-tuc-su-kien/2024/lac-quan-tai-chinh/</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Slogan đề xuất</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Hội đồng Thành viên</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/hoi-dong-thanh-vien/</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Danh sách HĐTV</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Ban Điều hành</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/ve-chung-toi/hoi-dong-thanh-vien/ban-dieu-hanh/</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>Danh sách Ban Điều hành</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Chương trình khuyến mại 2025</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sunlife.com.vn/vn/dich-vu-khach-hang/chuong-trinh-khuyen-mai/2025/</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Trang có liệt kê kênh social chính thức (Facebook, Youtube, Instagram, Zalo OA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Facebook chính thức</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/SunLifeVietnam</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Link social; username đề xuất; logo/ảnh bìa hiện tại</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Youtube chính thức</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/c/SunLifeVietnam</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Link social</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Instagram chính thức</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/sunlifevn/</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Link social</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Wikipedia – Postal codes in Vietnam</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Postal_codes_in_Vietnam</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Zipcode (nguồn ngoài website KH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>GHTK – Mã ZIP TP.HCM</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>https://ghtk.vn/blog/ma-zip-thanh-pho-ho-chi-minh/</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>Zipcode (nguồn ngoài website KH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Ghi chú: hashtag do team SEO đề xuất, không có nguồn. Website KH không có mục Giá trị cốt lõi, Tầm nhìn – Sứ mệnh, Khách hàng nổi bật.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>